<commit_message>
#56 Updated BOM Node Design.
</commit_message>
<xml_diff>
--- a/Deliverable/BOM/Client_BOM_Ezlo_Voice_Assistant_Node.xlsx
+++ b/Deliverable/BOM/Client_BOM_Ezlo_Voice_Assistant_Node.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\GitHub\Ezlo-VoiceAssistant\Deliverable\BOM\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{40436283-10BE-4FA0-8D93-92FEC44680EF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{24AAC17F-509A-45B8-9024-664000EBFDBE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="1170" yWindow="840" windowWidth="11790" windowHeight="15360" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -30,7 +30,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="634" uniqueCount="346">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="566" uniqueCount="345">
   <si>
     <t>Component list</t>
   </si>
@@ -1037,9 +1037,6 @@
     <t>MOQ (10 Boards)</t>
   </si>
   <si>
-    <t>Links</t>
-  </si>
-  <si>
     <t>Unit Cost (10 Boards)</t>
   </si>
   <si>
@@ -1055,9 +1052,6 @@
     <t>LY68L6400SLIT</t>
   </si>
   <si>
-    <t>Self Supplier</t>
-  </si>
-  <si>
     <t>Bill of Materials for Project [Node_Design]</t>
   </si>
   <si>
@@ -1068,6 +1062,9 @@
   </si>
   <si>
     <t>R20,R30</t>
+  </si>
+  <si>
+    <t>Quantity (10 Boards)</t>
   </si>
 </sst>
 </file>
@@ -1079,7 +1076,7 @@
     <numFmt numFmtId="165" formatCode="&quot;$&quot;#,##0.0000"/>
     <numFmt numFmtId="166" formatCode="&quot;$&quot;#,##0.00"/>
   </numFmts>
-  <fonts count="25" x14ac:knownFonts="1">
+  <fonts count="24" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -1091,6 +1088,7 @@
       <sz val="10"/>
       <color indexed="13"/>
       <name val="Arial"/>
+      <family val="2"/>
     </font>
     <font>
       <b/>
@@ -1225,14 +1223,6 @@
       <scheme val="minor"/>
     </font>
     <font>
-      <u/>
-      <sz val="11"/>
-      <color theme="10"/>
-      <name val="Calibri"/>
-      <family val="2"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
       <b/>
       <sz val="14"/>
       <name val="Calibri"/>
@@ -1287,7 +1277,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="21">
+  <borders count="22">
     <border>
       <left/>
       <right/>
@@ -1523,12 +1513,26 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left style="medium">
+        <color indexed="64"/>
+      </left>
+      <right style="medium">
+        <color indexed="64"/>
+      </right>
+      <top style="medium">
+        <color indexed="64"/>
+      </top>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
-  <cellStyleXfs count="2">
+  <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
-    <xf numFmtId="0" fontId="21" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="82">
+  <cellXfs count="81">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
@@ -1688,15 +1692,9 @@
     <xf numFmtId="0" fontId="20" fillId="2" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="21" fillId="2" borderId="15" xfId="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="165" fontId="17" fillId="2" borderId="15" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="21" fillId="4" borderId="16" xfId="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="165" fontId="17" fillId="4" borderId="16" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
@@ -1709,34 +1707,37 @@
     <xf numFmtId="0" fontId="17" fillId="4" borderId="20" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="22" fillId="2" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="23" fillId="2" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="24" fillId="2" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="23" fillId="2" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="24" fillId="2" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="22" fillId="4" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="23" fillId="4" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="24" fillId="4" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="23" fillId="4" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="24" fillId="4" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="165" fontId="23" fillId="2" borderId="15" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="165" fontId="24" fillId="2" borderId="15" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="165" fontId="24" fillId="4" borderId="16" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="165" fontId="23" fillId="4" borderId="16" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="17" fillId="2" borderId="21" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
@@ -1746,17 +1747,16 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="22" fillId="3" borderId="18" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+    <xf numFmtId="0" fontId="21" fillId="3" borderId="18" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center" vertical="top"/>
       <protection locked="0"/>
     </xf>
-    <xf numFmtId="0" fontId="22" fillId="3" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+    <xf numFmtId="0" fontId="21" fillId="3" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center" vertical="top"/>
       <protection locked="0"/>
     </xf>
   </cellXfs>
-  <cellStyles count="2">
-    <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
+  <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
@@ -2109,8 +2109,8 @@
     <col min="9" max="9" width="21.42578125" bestFit="1" customWidth="1"/>
     <col min="10" max="10" width="9" bestFit="1" customWidth="1"/>
     <col min="11" max="11" width="8.7109375" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="16.140625" bestFit="1" customWidth="1"/>
-    <col min="13" max="13" width="8.42578125" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="19.28515625" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="16.140625" bestFit="1" customWidth="1"/>
     <col min="14" max="14" width="19.7109375" bestFit="1" customWidth="1"/>
     <col min="15" max="15" width="20.28515625" bestFit="1" customWidth="1"/>
     <col min="16" max="16" width="29.42578125" customWidth="1"/>
@@ -2126,13 +2126,13 @@
       <c r="G1" s="2"/>
       <c r="H1" s="2"/>
       <c r="I1" s="2"/>
-      <c r="J1" s="77"/>
-      <c r="K1" s="77"/>
-      <c r="L1" s="77"/>
-      <c r="M1" s="77"/>
-      <c r="N1" s="77"/>
-      <c r="O1" s="77"/>
-      <c r="P1" s="77"/>
+      <c r="J1" s="76"/>
+      <c r="K1" s="76"/>
+      <c r="L1" s="76"/>
+      <c r="M1" s="76"/>
+      <c r="N1" s="76"/>
+      <c r="O1" s="76"/>
+      <c r="P1" s="76"/>
     </row>
     <row r="2" spans="1:22" ht="32.25" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A2" s="1"/>
@@ -2143,7 +2143,7 @@
       </c>
       <c r="E2" s="10"/>
       <c r="F2" s="51" t="s">
-        <v>342</v>
+        <v>340</v>
       </c>
       <c r="G2" s="11"/>
       <c r="H2" s="11"/>
@@ -2165,7 +2165,7 @@
       </c>
       <c r="E3" s="12"/>
       <c r="F3" s="52" t="s">
-        <v>343</v>
+        <v>341</v>
       </c>
       <c r="G3" s="12"/>
       <c r="H3" s="12"/>
@@ -2176,7 +2176,7 @@
       <c r="M3" s="4"/>
       <c r="N3" s="4"/>
       <c r="O3" s="4"/>
-      <c r="P3" s="78"/>
+      <c r="P3" s="77"/>
     </row>
     <row r="4" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A4" s="1"/>
@@ -2187,7 +2187,7 @@
       </c>
       <c r="E4" s="12"/>
       <c r="F4" s="53" t="s">
-        <v>343</v>
+        <v>341</v>
       </c>
       <c r="G4" s="13"/>
       <c r="H4" s="13"/>
@@ -2198,7 +2198,7 @@
       <c r="M4" s="5"/>
       <c r="N4" s="5"/>
       <c r="O4" s="5"/>
-      <c r="P4" s="79"/>
+      <c r="P4" s="78"/>
     </row>
     <row r="5" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A5" s="1"/>
@@ -2220,7 +2220,7 @@
       <c r="M5" s="5"/>
       <c r="N5" s="5"/>
       <c r="O5" s="5"/>
-      <c r="P5" s="79"/>
+      <c r="P5" s="78"/>
     </row>
     <row r="6" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A6" s="1"/>
@@ -2238,7 +2238,7 @@
       <c r="M6" s="5"/>
       <c r="N6" s="5"/>
       <c r="O6" s="5"/>
-      <c r="P6" s="79"/>
+      <c r="P6" s="78"/>
     </row>
     <row r="7" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A7" s="1"/>
@@ -2256,7 +2256,7 @@
       <c r="M7" s="7"/>
       <c r="N7" s="7"/>
       <c r="O7" s="7"/>
-      <c r="P7" s="79"/>
+      <c r="P7" s="78"/>
     </row>
     <row r="8" spans="1:22" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A8" s="1"/>
@@ -2274,7 +2274,7 @@
       <c r="M8" s="7"/>
       <c r="N8" s="7"/>
       <c r="O8" s="7"/>
-      <c r="P8" s="79"/>
+      <c r="P8" s="78"/>
     </row>
     <row r="9" spans="1:22" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A9" s="1"/>
@@ -2309,22 +2309,22 @@
         <v>301</v>
       </c>
       <c r="L9" s="29" t="s">
+        <v>344</v>
+      </c>
+      <c r="M9" s="29" t="s">
         <v>334</v>
       </c>
-      <c r="M9" s="29" t="s">
+      <c r="N9" s="29" t="s">
         <v>335</v>
       </c>
-      <c r="N9" s="29" t="s">
+      <c r="O9" s="29" t="s">
         <v>336</v>
       </c>
-      <c r="O9" s="29" t="s">
-        <v>337</v>
-      </c>
       <c r="P9" s="29" t="s">
-        <v>344</v>
-      </c>
-    </row>
-    <row r="10" spans="1:22" ht="30.75" thickBot="1" x14ac:dyDescent="0.3">
+        <v>342</v>
+      </c>
+    </row>
+    <row r="10" spans="1:22" ht="24.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A10" s="1"/>
       <c r="B10" s="50">
         <f>ROW(B10) - ROW($B$9)</f>
@@ -2357,28 +2357,29 @@
       <c r="K10" s="36">
         <v>13</v>
       </c>
-      <c r="L10" s="36">
+      <c r="L10" s="75">
+        <f>K10*10</f>
+        <v>130</v>
+      </c>
+      <c r="M10" s="36">
         <v>200</v>
       </c>
-      <c r="M10" s="60" t="s">
-        <v>341</v>
-      </c>
-      <c r="N10" s="61">
+      <c r="N10" s="60">
         <v>0.20290000000000002</v>
       </c>
-      <c r="O10" s="61">
-        <f>N10*L10</f>
+      <c r="O10" s="60">
+        <f t="shared" ref="O10:O44" si="0">N10*M10</f>
         <v>40.580000000000005</v>
       </c>
       <c r="P10" s="36"/>
-      <c r="R10" s="75"/>
-      <c r="U10" s="75"/>
-      <c r="V10" s="76"/>
+      <c r="R10" s="73"/>
+      <c r="U10" s="73"/>
+      <c r="V10" s="74"/>
     </row>
     <row r="11" spans="1:22" ht="36.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A11" s="1"/>
       <c r="B11" s="50">
-        <f t="shared" ref="B11:B77" si="0">ROW(B11) - ROW($B$9)</f>
+        <f t="shared" ref="B11:B77" si="1">ROW(B11) - ROW($B$9)</f>
         <v>2</v>
       </c>
       <c r="C11" s="56" t="s">
@@ -2409,22 +2410,23 @@
         <v>4</v>
       </c>
       <c r="L11" s="38">
+        <f t="shared" ref="L11:L74" si="2">K11*10</f>
+        <v>40</v>
+      </c>
+      <c r="M11" s="38">
         <v>50</v>
       </c>
-      <c r="M11" s="62" t="s">
-        <v>341</v>
-      </c>
-      <c r="N11" s="63">
+      <c r="N11" s="61">
         <v>0.18859999999999999</v>
       </c>
-      <c r="O11" s="63">
-        <f t="shared" ref="O11:O74" si="1">N11*L11</f>
+      <c r="O11" s="61">
+        <f t="shared" si="0"/>
         <v>9.43</v>
       </c>
       <c r="P11" s="38"/>
-      <c r="R11" s="75"/>
-      <c r="U11" s="75"/>
-      <c r="V11" s="76"/>
+      <c r="R11" s="73"/>
+      <c r="U11" s="73"/>
+      <c r="V11" s="74"/>
     </row>
     <row r="12" spans="1:22" ht="48.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A12" s="1"/>
@@ -2460,27 +2462,28 @@
         <v>2</v>
       </c>
       <c r="L12" s="36">
+        <f t="shared" si="2"/>
+        <v>20</v>
+      </c>
+      <c r="M12" s="36">
         <v>22</v>
       </c>
-      <c r="M12" s="60" t="s">
-        <v>341</v>
-      </c>
-      <c r="N12" s="61">
+      <c r="N12" s="60">
         <v>0.58550000000000002</v>
       </c>
-      <c r="O12" s="61">
-        <f t="shared" si="1"/>
+      <c r="O12" s="60">
+        <f t="shared" si="0"/>
         <v>12.881</v>
       </c>
       <c r="P12" s="36"/>
-      <c r="R12" s="75"/>
-      <c r="U12" s="75"/>
-      <c r="V12" s="76"/>
-    </row>
-    <row r="13" spans="1:22" ht="30.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="R12" s="73"/>
+      <c r="U12" s="73"/>
+      <c r="V12" s="74"/>
+    </row>
+    <row r="13" spans="1:22" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A13" s="1"/>
       <c r="B13" s="50">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>4</v>
       </c>
       <c r="C13" s="56" t="s">
@@ -2511,24 +2514,25 @@
         <v>1</v>
       </c>
       <c r="L13" s="38">
+        <f t="shared" si="2"/>
+        <v>10</v>
+      </c>
+      <c r="M13" s="38">
         <v>100</v>
       </c>
-      <c r="M13" s="62" t="s">
-        <v>341</v>
-      </c>
-      <c r="N13" s="63">
+      <c r="N13" s="61">
         <v>0.10250000000000001</v>
       </c>
-      <c r="O13" s="63">
-        <f t="shared" si="1"/>
+      <c r="O13" s="61">
+        <f t="shared" si="0"/>
         <v>10.25</v>
       </c>
       <c r="P13" s="38"/>
-      <c r="R13" s="75"/>
-      <c r="U13" s="75"/>
-      <c r="V13" s="76"/>
-    </row>
-    <row r="14" spans="1:22" ht="30.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="R13" s="73"/>
+      <c r="U13" s="73"/>
+      <c r="V13" s="74"/>
+    </row>
+    <row r="14" spans="1:22" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A14" s="1"/>
       <c r="B14" s="50">
         <f>ROW(B14) - ROW($B$9)</f>
@@ -2562,27 +2566,28 @@
         <v>1</v>
       </c>
       <c r="L14" s="36">
+        <f t="shared" si="2"/>
+        <v>10</v>
+      </c>
+      <c r="M14" s="36">
         <v>100</v>
       </c>
-      <c r="M14" s="60" t="s">
-        <v>341</v>
-      </c>
-      <c r="N14" s="61">
+      <c r="N14" s="60">
         <v>0.10310000000000001</v>
       </c>
-      <c r="O14" s="61">
-        <f t="shared" si="1"/>
+      <c r="O14" s="60">
+        <f t="shared" si="0"/>
         <v>10.31</v>
       </c>
       <c r="P14" s="36"/>
-      <c r="R14" s="75"/>
-      <c r="U14" s="75"/>
-      <c r="V14" s="76"/>
-    </row>
-    <row r="15" spans="1:22" ht="30.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="R14" s="73"/>
+      <c r="U14" s="73"/>
+      <c r="V14" s="74"/>
+    </row>
+    <row r="15" spans="1:22" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A15" s="1"/>
       <c r="B15" s="50">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>6</v>
       </c>
       <c r="C15" s="56" t="s">
@@ -2613,24 +2618,25 @@
         <v>2</v>
       </c>
       <c r="L15" s="38">
+        <f t="shared" si="2"/>
+        <v>20</v>
+      </c>
+      <c r="M15" s="38">
         <v>40</v>
       </c>
-      <c r="M15" s="62" t="s">
-        <v>341</v>
-      </c>
-      <c r="N15" s="63">
+      <c r="N15" s="61">
         <v>0.11420000000000001</v>
       </c>
-      <c r="O15" s="63">
-        <f t="shared" si="1"/>
+      <c r="O15" s="61">
+        <f t="shared" si="0"/>
         <v>4.5680000000000005</v>
       </c>
       <c r="P15" s="38"/>
-      <c r="R15" s="75"/>
-      <c r="U15" s="75"/>
-      <c r="V15" s="76"/>
-    </row>
-    <row r="16" spans="1:22" ht="30.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="R15" s="73"/>
+      <c r="U15" s="73"/>
+      <c r="V15" s="74"/>
+    </row>
+    <row r="16" spans="1:22" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A16" s="1"/>
       <c r="B16" s="50">
         <f>ROW(B16) - ROW($B$9)</f>
@@ -2664,27 +2670,28 @@
         <v>2</v>
       </c>
       <c r="L16" s="36">
+        <f t="shared" si="2"/>
+        <v>20</v>
+      </c>
+      <c r="M16" s="36">
         <v>100</v>
       </c>
-      <c r="M16" s="60" t="s">
-        <v>341</v>
-      </c>
-      <c r="N16" s="61">
+      <c r="N16" s="60">
         <v>0.10100000000000001</v>
       </c>
-      <c r="O16" s="61">
-        <f t="shared" si="1"/>
+      <c r="O16" s="60">
+        <f t="shared" si="0"/>
         <v>10.100000000000001</v>
       </c>
       <c r="P16" s="36"/>
-      <c r="R16" s="75"/>
-      <c r="U16" s="75"/>
-      <c r="V16" s="76"/>
-    </row>
-    <row r="17" spans="1:22" ht="30.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="R16" s="73"/>
+      <c r="U16" s="73"/>
+      <c r="V16" s="74"/>
+    </row>
+    <row r="17" spans="1:22" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A17" s="1"/>
       <c r="B17" s="50">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>8</v>
       </c>
       <c r="C17" s="56" t="s">
@@ -2715,24 +2722,25 @@
         <v>1</v>
       </c>
       <c r="L17" s="38">
+        <f t="shared" si="2"/>
+        <v>10</v>
+      </c>
+      <c r="M17" s="38">
         <v>100</v>
       </c>
-      <c r="M17" s="62" t="s">
-        <v>341</v>
-      </c>
-      <c r="N17" s="63">
+      <c r="N17" s="61">
         <v>0.1032</v>
       </c>
-      <c r="O17" s="63">
-        <f t="shared" si="1"/>
+      <c r="O17" s="61">
+        <f t="shared" si="0"/>
         <v>10.32</v>
       </c>
       <c r="P17" s="38"/>
-      <c r="R17" s="75"/>
-      <c r="U17" s="75"/>
-      <c r="V17" s="76"/>
-    </row>
-    <row r="18" spans="1:22" ht="30.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="R17" s="73"/>
+      <c r="U17" s="73"/>
+      <c r="V17" s="74"/>
+    </row>
+    <row r="18" spans="1:22" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A18" s="1"/>
       <c r="B18" s="50">
         <f>ROW(B18) - ROW($B$9)</f>
@@ -2766,27 +2774,28 @@
         <v>1</v>
       </c>
       <c r="L18" s="36">
+        <f t="shared" si="2"/>
+        <v>10</v>
+      </c>
+      <c r="M18" s="36">
         <v>20</v>
       </c>
-      <c r="M18" s="60" t="s">
-        <v>341</v>
-      </c>
-      <c r="N18" s="61">
+      <c r="N18" s="60">
         <v>0.1179</v>
       </c>
-      <c r="O18" s="61">
-        <f t="shared" si="1"/>
+      <c r="O18" s="60">
+        <f t="shared" si="0"/>
         <v>2.3580000000000001</v>
       </c>
       <c r="P18" s="36"/>
-      <c r="R18" s="75"/>
-      <c r="U18" s="75"/>
-      <c r="V18" s="76"/>
-    </row>
-    <row r="19" spans="1:22" ht="30.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="R18" s="73"/>
+      <c r="U18" s="73"/>
+      <c r="V18" s="74"/>
+    </row>
+    <row r="19" spans="1:22" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A19" s="1"/>
       <c r="B19" s="50">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>10</v>
       </c>
       <c r="C19" s="56" t="s">
@@ -2817,24 +2826,25 @@
         <v>1</v>
       </c>
       <c r="L19" s="38">
+        <f t="shared" si="2"/>
+        <v>10</v>
+      </c>
+      <c r="M19" s="38">
         <v>100</v>
       </c>
-      <c r="M19" s="62" t="s">
-        <v>341</v>
-      </c>
-      <c r="N19" s="63">
+      <c r="N19" s="61">
         <v>0.10200000000000001</v>
       </c>
-      <c r="O19" s="63">
-        <f t="shared" si="1"/>
+      <c r="O19" s="61">
+        <f t="shared" si="0"/>
         <v>10.200000000000001</v>
       </c>
       <c r="P19" s="38"/>
-      <c r="R19" s="75"/>
-      <c r="U19" s="75"/>
-      <c r="V19" s="76"/>
-    </row>
-    <row r="20" spans="1:22" ht="30.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="R19" s="73"/>
+      <c r="U19" s="73"/>
+      <c r="V19" s="74"/>
+    </row>
+    <row r="20" spans="1:22" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A20" s="1"/>
       <c r="B20" s="50">
         <f>ROW(B20) - ROW($B$9)</f>
@@ -2868,27 +2878,28 @@
         <v>1</v>
       </c>
       <c r="L20" s="36">
+        <f t="shared" si="2"/>
+        <v>10</v>
+      </c>
+      <c r="M20" s="36">
         <v>100</v>
       </c>
-      <c r="M20" s="60" t="s">
-        <v>341</v>
-      </c>
-      <c r="N20" s="61">
+      <c r="N20" s="60">
         <v>0.10210000000000001</v>
       </c>
-      <c r="O20" s="61">
-        <f t="shared" si="1"/>
+      <c r="O20" s="60">
+        <f t="shared" si="0"/>
         <v>10.210000000000001</v>
       </c>
       <c r="P20" s="36"/>
-      <c r="R20" s="75"/>
-      <c r="U20" s="75"/>
-      <c r="V20" s="76"/>
-    </row>
-    <row r="21" spans="1:22" ht="30.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="R20" s="73"/>
+      <c r="U20" s="73"/>
+      <c r="V20" s="74"/>
+    </row>
+    <row r="21" spans="1:22" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A21" s="1"/>
       <c r="B21" s="50">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>12</v>
       </c>
       <c r="C21" s="56" t="s">
@@ -2919,24 +2930,25 @@
         <v>8</v>
       </c>
       <c r="L21" s="38">
+        <f t="shared" si="2"/>
+        <v>80</v>
+      </c>
+      <c r="M21" s="38">
         <v>100</v>
       </c>
-      <c r="M21" s="62" t="s">
-        <v>341</v>
-      </c>
-      <c r="N21" s="63">
+      <c r="N21" s="61">
         <v>0.10740000000000001</v>
       </c>
-      <c r="O21" s="63">
-        <f t="shared" si="1"/>
+      <c r="O21" s="61">
+        <f t="shared" si="0"/>
         <v>10.74</v>
       </c>
       <c r="P21" s="38"/>
-      <c r="R21" s="75"/>
-      <c r="U21" s="75"/>
-      <c r="V21" s="76"/>
-    </row>
-    <row r="22" spans="1:22" ht="30.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="R21" s="73"/>
+      <c r="U21" s="73"/>
+      <c r="V21" s="74"/>
+    </row>
+    <row r="22" spans="1:22" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A22" s="1"/>
       <c r="B22" s="50">
         <f>ROW(B22) - ROW($B$9)</f>
@@ -2970,27 +2982,28 @@
         <v>2</v>
       </c>
       <c r="L22" s="36">
+        <f t="shared" si="2"/>
+        <v>20</v>
+      </c>
+      <c r="M22" s="36">
         <v>100</v>
       </c>
-      <c r="M22" s="60" t="s">
-        <v>341</v>
-      </c>
-      <c r="N22" s="61">
+      <c r="N22" s="60">
         <v>0.1028</v>
       </c>
-      <c r="O22" s="61">
-        <f t="shared" si="1"/>
+      <c r="O22" s="60">
+        <f t="shared" si="0"/>
         <v>10.280000000000001</v>
       </c>
       <c r="P22" s="36"/>
-      <c r="R22" s="75"/>
-      <c r="U22" s="75"/>
-      <c r="V22" s="76"/>
-    </row>
-    <row r="23" spans="1:22" ht="30.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="R22" s="73"/>
+      <c r="U22" s="73"/>
+      <c r="V22" s="74"/>
+    </row>
+    <row r="23" spans="1:22" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A23" s="1"/>
       <c r="B23" s="50">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>14</v>
       </c>
       <c r="C23" s="56" t="s">
@@ -3021,24 +3034,25 @@
         <v>2</v>
       </c>
       <c r="L23" s="38">
+        <f t="shared" si="2"/>
+        <v>20</v>
+      </c>
+      <c r="M23" s="38">
         <v>22</v>
       </c>
-      <c r="M23" s="62" t="s">
-        <v>341</v>
-      </c>
-      <c r="N23" s="63">
+      <c r="N23" s="61">
         <v>0.29010000000000002</v>
       </c>
-      <c r="O23" s="63">
-        <f t="shared" si="1"/>
+      <c r="O23" s="61">
+        <f t="shared" si="0"/>
         <v>6.382200000000001</v>
       </c>
       <c r="P23" s="38"/>
-      <c r="R23" s="75"/>
-      <c r="U23" s="75"/>
-      <c r="V23" s="76"/>
-    </row>
-    <row r="24" spans="1:22" ht="30.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="R23" s="73"/>
+      <c r="U23" s="73"/>
+      <c r="V23" s="74"/>
+    </row>
+    <row r="24" spans="1:22" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A24" s="1"/>
       <c r="B24" s="50">
         <f>ROW(B24) - ROW($B$9)</f>
@@ -3072,27 +3086,28 @@
         <v>2</v>
       </c>
       <c r="L24" s="36">
+        <f t="shared" si="2"/>
+        <v>20</v>
+      </c>
+      <c r="M24" s="36">
         <v>40</v>
       </c>
-      <c r="M24" s="60" t="s">
-        <v>341</v>
-      </c>
-      <c r="N24" s="61">
+      <c r="N24" s="60">
         <v>0.129</v>
       </c>
-      <c r="O24" s="61">
-        <f t="shared" si="1"/>
+      <c r="O24" s="60">
+        <f t="shared" si="0"/>
         <v>5.16</v>
       </c>
       <c r="P24" s="36"/>
-      <c r="R24" s="75"/>
-      <c r="U24" s="75"/>
-      <c r="V24" s="76"/>
-    </row>
-    <row r="25" spans="1:22" ht="30.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="R24" s="73"/>
+      <c r="U24" s="73"/>
+      <c r="V24" s="74"/>
+    </row>
+    <row r="25" spans="1:22" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A25" s="1"/>
       <c r="B25" s="50">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>16</v>
       </c>
       <c r="C25" s="56" t="s">
@@ -3123,24 +3138,25 @@
         <v>2</v>
       </c>
       <c r="L25" s="38">
+        <f t="shared" si="2"/>
+        <v>20</v>
+      </c>
+      <c r="M25" s="38">
         <v>50</v>
       </c>
-      <c r="M25" s="62" t="s">
-        <v>341</v>
-      </c>
-      <c r="N25" s="63">
+      <c r="N25" s="61">
         <v>0.1119</v>
       </c>
-      <c r="O25" s="63">
-        <f t="shared" si="1"/>
+      <c r="O25" s="61">
+        <f t="shared" si="0"/>
         <v>5.5949999999999998</v>
       </c>
       <c r="P25" s="38"/>
-      <c r="R25" s="75"/>
-      <c r="U25" s="75"/>
-      <c r="V25" s="76"/>
-    </row>
-    <row r="26" spans="1:22" ht="30.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="R25" s="73"/>
+      <c r="U25" s="73"/>
+      <c r="V25" s="74"/>
+    </row>
+    <row r="26" spans="1:22" ht="24.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A26" s="1"/>
       <c r="B26" s="50">
         <f>ROW(B26) - ROW($B$9)</f>
@@ -3174,27 +3190,28 @@
         <v>13</v>
       </c>
       <c r="L26" s="36">
+        <f t="shared" si="2"/>
+        <v>130</v>
+      </c>
+      <c r="M26" s="36">
         <v>150</v>
       </c>
-      <c r="M26" s="60" t="s">
-        <v>341</v>
-      </c>
-      <c r="N26" s="61">
+      <c r="N26" s="60">
         <v>0.1042</v>
       </c>
-      <c r="O26" s="61">
-        <f t="shared" si="1"/>
+      <c r="O26" s="60">
+        <f t="shared" si="0"/>
         <v>15.63</v>
       </c>
       <c r="P26" s="36"/>
-      <c r="R26" s="75"/>
-      <c r="U26" s="75"/>
-      <c r="V26" s="76"/>
-    </row>
-    <row r="27" spans="1:22" ht="30.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="R26" s="73"/>
+      <c r="U26" s="73"/>
+      <c r="V26" s="74"/>
+    </row>
+    <row r="27" spans="1:22" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A27" s="1"/>
       <c r="B27" s="50">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>18</v>
       </c>
       <c r="C27" s="56" t="s">
@@ -3225,24 +3242,25 @@
         <v>1</v>
       </c>
       <c r="L27" s="38">
+        <f t="shared" si="2"/>
+        <v>10</v>
+      </c>
+      <c r="M27" s="38">
         <v>50</v>
       </c>
-      <c r="M27" s="62" t="s">
-        <v>341</v>
-      </c>
-      <c r="N27" s="63">
+      <c r="N27" s="61">
         <v>0.1067</v>
       </c>
-      <c r="O27" s="63">
-        <f t="shared" si="1"/>
+      <c r="O27" s="61">
+        <f t="shared" si="0"/>
         <v>5.335</v>
       </c>
       <c r="P27" s="38"/>
-      <c r="R27" s="75"/>
-      <c r="U27" s="75"/>
-      <c r="V27" s="76"/>
-    </row>
-    <row r="28" spans="1:22" ht="30.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="R27" s="73"/>
+      <c r="U27" s="73"/>
+      <c r="V27" s="74"/>
+    </row>
+    <row r="28" spans="1:22" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A28" s="1"/>
       <c r="B28" s="50">
         <f>ROW(B28) - ROW($B$9)</f>
@@ -3276,27 +3294,28 @@
         <v>1</v>
       </c>
       <c r="L28" s="36">
+        <f t="shared" si="2"/>
+        <v>10</v>
+      </c>
+      <c r="M28" s="36">
         <v>50</v>
       </c>
-      <c r="M28" s="60" t="s">
-        <v>341</v>
-      </c>
-      <c r="N28" s="61">
+      <c r="N28" s="60">
         <v>0.1052</v>
       </c>
-      <c r="O28" s="61">
-        <f t="shared" si="1"/>
+      <c r="O28" s="60">
+        <f t="shared" si="0"/>
         <v>5.26</v>
       </c>
       <c r="P28" s="36"/>
-      <c r="R28" s="75"/>
-      <c r="U28" s="75"/>
-      <c r="V28" s="76"/>
-    </row>
-    <row r="29" spans="1:22" ht="30.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="R28" s="73"/>
+      <c r="U28" s="73"/>
+      <c r="V28" s="74"/>
+    </row>
+    <row r="29" spans="1:22" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A29" s="1"/>
       <c r="B29" s="50">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>20</v>
       </c>
       <c r="C29" s="56" t="s">
@@ -3327,24 +3346,25 @@
         <v>6</v>
       </c>
       <c r="L29" s="38">
+        <f t="shared" si="2"/>
+        <v>60</v>
+      </c>
+      <c r="M29" s="38">
         <v>100</v>
       </c>
-      <c r="M29" s="62" t="s">
-        <v>341</v>
-      </c>
-      <c r="N29" s="63">
+      <c r="N29" s="61">
         <v>0.10450000000000001</v>
       </c>
-      <c r="O29" s="63">
-        <f t="shared" si="1"/>
+      <c r="O29" s="61">
+        <f t="shared" si="0"/>
         <v>10.450000000000001</v>
       </c>
       <c r="P29" s="38"/>
-      <c r="R29" s="75"/>
-      <c r="U29" s="75"/>
-      <c r="V29" s="76"/>
-    </row>
-    <row r="30" spans="1:22" ht="30.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="R29" s="73"/>
+      <c r="U29" s="73"/>
+      <c r="V29" s="74"/>
+    </row>
+    <row r="30" spans="1:22" ht="24.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A30" s="1"/>
       <c r="B30" s="50">
         <f>ROW(B30) - ROW($B$9)</f>
@@ -3378,27 +3398,28 @@
         <v>2</v>
       </c>
       <c r="L30" s="36">
+        <f t="shared" si="2"/>
+        <v>20</v>
+      </c>
+      <c r="M30" s="36">
         <v>40</v>
       </c>
-      <c r="M30" s="60" t="s">
-        <v>341</v>
-      </c>
-      <c r="N30" s="61">
+      <c r="N30" s="60">
         <v>0.12520000000000001</v>
       </c>
-      <c r="O30" s="61">
-        <f t="shared" si="1"/>
+      <c r="O30" s="60">
+        <f t="shared" si="0"/>
         <v>5.008</v>
       </c>
       <c r="P30" s="36"/>
-      <c r="R30" s="75"/>
-      <c r="U30" s="75"/>
-      <c r="V30" s="76"/>
-    </row>
-    <row r="31" spans="1:22" ht="30.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="R30" s="73"/>
+      <c r="U30" s="73"/>
+      <c r="V30" s="74"/>
+    </row>
+    <row r="31" spans="1:22" ht="24.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A31" s="1"/>
       <c r="B31" s="50">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>22</v>
       </c>
       <c r="C31" s="56" t="s">
@@ -3429,24 +3450,25 @@
         <v>1</v>
       </c>
       <c r="L31" s="38">
+        <f t="shared" si="2"/>
+        <v>10</v>
+      </c>
+      <c r="M31" s="38">
         <v>20</v>
       </c>
-      <c r="M31" s="62" t="s">
-        <v>341</v>
-      </c>
-      <c r="N31" s="63">
+      <c r="N31" s="61">
         <v>0.14900000000000002</v>
       </c>
-      <c r="O31" s="63">
-        <f t="shared" si="1"/>
+      <c r="O31" s="61">
+        <f t="shared" si="0"/>
         <v>2.9800000000000004</v>
       </c>
       <c r="P31" s="38"/>
-      <c r="R31" s="75"/>
-      <c r="U31" s="75"/>
-      <c r="V31" s="76"/>
-    </row>
-    <row r="32" spans="1:22" ht="30.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="R31" s="73"/>
+      <c r="U31" s="73"/>
+      <c r="V31" s="74"/>
+    </row>
+    <row r="32" spans="1:22" ht="24.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A32" s="1"/>
       <c r="B32" s="50">
         <f>ROW(B32) - ROW($B$9)</f>
@@ -3480,27 +3502,28 @@
         <v>1</v>
       </c>
       <c r="L32" s="36">
+        <f t="shared" si="2"/>
+        <v>10</v>
+      </c>
+      <c r="M32" s="36">
         <v>50</v>
       </c>
-      <c r="M32" s="60" t="s">
-        <v>341</v>
-      </c>
-      <c r="N32" s="61">
+      <c r="N32" s="60">
         <v>0.11950000000000001</v>
       </c>
-      <c r="O32" s="61">
-        <f t="shared" si="1"/>
+      <c r="O32" s="60">
+        <f t="shared" si="0"/>
         <v>5.9750000000000005</v>
       </c>
       <c r="P32" s="36"/>
-      <c r="R32" s="75"/>
-      <c r="U32" s="75"/>
-      <c r="V32" s="76"/>
-    </row>
-    <row r="33" spans="1:22" ht="30.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="R32" s="73"/>
+      <c r="U32" s="73"/>
+      <c r="V32" s="74"/>
+    </row>
+    <row r="33" spans="1:22" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A33" s="1"/>
       <c r="B33" s="50">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>24</v>
       </c>
       <c r="C33" s="56" t="s">
@@ -3531,24 +3554,25 @@
         <v>1</v>
       </c>
       <c r="L33" s="38">
+        <f t="shared" si="2"/>
+        <v>10</v>
+      </c>
+      <c r="M33" s="38">
         <v>15</v>
       </c>
-      <c r="M33" s="62" t="s">
-        <v>341</v>
-      </c>
-      <c r="N33" s="63">
+      <c r="N33" s="61">
         <v>0.1875</v>
       </c>
-      <c r="O33" s="63">
-        <f t="shared" si="1"/>
+      <c r="O33" s="61">
+        <f t="shared" si="0"/>
         <v>2.8125</v>
       </c>
       <c r="P33" s="38"/>
-      <c r="R33" s="75"/>
-      <c r="U33" s="75"/>
-      <c r="V33" s="76"/>
-    </row>
-    <row r="34" spans="1:22" ht="30.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="R33" s="73"/>
+      <c r="U33" s="73"/>
+      <c r="V33" s="74"/>
+    </row>
+    <row r="34" spans="1:22" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A34" s="1"/>
       <c r="B34" s="50">
         <f>ROW(B34) - ROW($B$9)</f>
@@ -3582,27 +3606,28 @@
         <v>1</v>
       </c>
       <c r="L34" s="36">
+        <f t="shared" si="2"/>
+        <v>10</v>
+      </c>
+      <c r="M34" s="36">
         <v>20</v>
       </c>
-      <c r="M34" s="60" t="s">
-        <v>341</v>
-      </c>
-      <c r="N34" s="61">
+      <c r="N34" s="60">
         <v>0.12560000000000002</v>
       </c>
-      <c r="O34" s="61">
-        <f t="shared" si="1"/>
+      <c r="O34" s="60">
+        <f t="shared" si="0"/>
         <v>2.5120000000000005</v>
       </c>
       <c r="P34" s="36"/>
-      <c r="R34" s="75"/>
-      <c r="U34" s="75"/>
-      <c r="V34" s="76"/>
+      <c r="R34" s="73"/>
+      <c r="U34" s="73"/>
+      <c r="V34" s="74"/>
     </row>
     <row r="35" spans="1:22" ht="36.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A35" s="1"/>
       <c r="B35" s="50">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>26</v>
       </c>
       <c r="C35" s="56" t="s">
@@ -3633,22 +3658,23 @@
         <v>1</v>
       </c>
       <c r="L35" s="38">
+        <f t="shared" si="2"/>
+        <v>10</v>
+      </c>
+      <c r="M35" s="38">
         <v>11</v>
       </c>
-      <c r="M35" s="62" t="s">
-        <v>341</v>
-      </c>
-      <c r="N35" s="63">
+      <c r="N35" s="61">
         <v>0.76449999999999996</v>
       </c>
-      <c r="O35" s="63">
-        <f t="shared" si="1"/>
+      <c r="O35" s="61">
+        <f t="shared" si="0"/>
         <v>8.4094999999999995</v>
       </c>
       <c r="P35" s="38"/>
-      <c r="R35" s="75"/>
-      <c r="U35" s="75"/>
-      <c r="V35" s="76"/>
+      <c r="R35" s="73"/>
+      <c r="U35" s="73"/>
+      <c r="V35" s="74"/>
     </row>
     <row r="36" spans="1:22" ht="36.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A36" s="1"/>
@@ -3684,27 +3710,28 @@
         <v>1</v>
       </c>
       <c r="L36" s="36">
+        <f t="shared" si="2"/>
+        <v>10</v>
+      </c>
+      <c r="M36" s="36">
         <v>12</v>
       </c>
-      <c r="M36" s="60" t="s">
-        <v>341</v>
-      </c>
-      <c r="N36" s="61">
+      <c r="N36" s="60">
         <v>0.5252</v>
       </c>
-      <c r="O36" s="61">
-        <f t="shared" si="1"/>
+      <c r="O36" s="60">
+        <f t="shared" si="0"/>
         <v>6.3024000000000004</v>
       </c>
       <c r="P36" s="36"/>
-      <c r="R36" s="75"/>
-      <c r="U36" s="75"/>
-      <c r="V36" s="76"/>
+      <c r="R36" s="73"/>
+      <c r="U36" s="73"/>
+      <c r="V36" s="74"/>
     </row>
     <row r="37" spans="1:22" ht="36.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A37" s="1"/>
       <c r="B37" s="50">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>28</v>
       </c>
       <c r="C37" s="56" t="s">
@@ -3735,24 +3762,25 @@
         <v>1</v>
       </c>
       <c r="L37" s="38">
+        <f t="shared" si="2"/>
+        <v>10</v>
+      </c>
+      <c r="M37" s="38">
         <v>12</v>
       </c>
-      <c r="M37" s="62" t="s">
-        <v>341</v>
-      </c>
-      <c r="N37" s="63">
+      <c r="N37" s="61">
         <v>0.26500000000000001</v>
       </c>
-      <c r="O37" s="63">
-        <f t="shared" si="1"/>
+      <c r="O37" s="61">
+        <f t="shared" si="0"/>
         <v>3.18</v>
       </c>
       <c r="P37" s="38"/>
-      <c r="R37" s="75"/>
-      <c r="U37" s="75"/>
-      <c r="V37" s="76"/>
-    </row>
-    <row r="38" spans="1:22" ht="30.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="R37" s="73"/>
+      <c r="U37" s="73"/>
+      <c r="V37" s="74"/>
+    </row>
+    <row r="38" spans="1:22" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A38" s="1"/>
       <c r="B38" s="50">
         <f>ROW(B38) - ROW($B$9)</f>
@@ -3786,27 +3814,28 @@
         <v>1</v>
       </c>
       <c r="L38" s="36">
+        <f t="shared" si="2"/>
+        <v>10</v>
+      </c>
+      <c r="M38" s="36">
         <v>50</v>
       </c>
-      <c r="M38" s="60" t="s">
-        <v>341</v>
-      </c>
-      <c r="N38" s="61">
+      <c r="N38" s="60">
         <v>0.10970000000000001</v>
       </c>
-      <c r="O38" s="61">
-        <f t="shared" si="1"/>
+      <c r="O38" s="60">
+        <f t="shared" si="0"/>
         <v>5.4850000000000003</v>
       </c>
       <c r="P38" s="36"/>
-      <c r="R38" s="75"/>
-      <c r="U38" s="75"/>
-      <c r="V38" s="76"/>
-    </row>
-    <row r="39" spans="1:22" ht="30.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="R38" s="73"/>
+      <c r="U38" s="73"/>
+      <c r="V38" s="74"/>
+    </row>
+    <row r="39" spans="1:22" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A39" s="1"/>
       <c r="B39" s="50">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>30</v>
       </c>
       <c r="C39" s="56" t="s">
@@ -3837,24 +3866,25 @@
         <v>2</v>
       </c>
       <c r="L39" s="38">
+        <f t="shared" si="2"/>
+        <v>20</v>
+      </c>
+      <c r="M39" s="38">
         <v>30</v>
       </c>
-      <c r="M39" s="62" t="s">
-        <v>341</v>
-      </c>
-      <c r="N39" s="63">
+      <c r="N39" s="61">
         <v>0.16450000000000001</v>
       </c>
-      <c r="O39" s="63">
-        <f t="shared" si="1"/>
+      <c r="O39" s="61">
+        <f t="shared" si="0"/>
         <v>4.9350000000000005</v>
       </c>
       <c r="P39" s="38"/>
-      <c r="R39" s="75"/>
-      <c r="U39" s="75"/>
-      <c r="V39" s="76"/>
-    </row>
-    <row r="40" spans="1:22" ht="30.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="R39" s="73"/>
+      <c r="U39" s="73"/>
+      <c r="V39" s="74"/>
+    </row>
+    <row r="40" spans="1:22" ht="24.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A40" s="1"/>
       <c r="B40" s="50">
         <f>ROW(B40) - ROW($B$9)</f>
@@ -3888,27 +3918,28 @@
         <v>1</v>
       </c>
       <c r="L40" s="36">
+        <f t="shared" si="2"/>
+        <v>10</v>
+      </c>
+      <c r="M40" s="36">
         <v>20</v>
       </c>
-      <c r="M40" s="60" t="s">
-        <v>341</v>
-      </c>
-      <c r="N40" s="61">
+      <c r="N40" s="60">
         <v>0.18590000000000001</v>
       </c>
-      <c r="O40" s="61">
-        <f t="shared" si="1"/>
+      <c r="O40" s="60">
+        <f t="shared" si="0"/>
         <v>3.718</v>
       </c>
       <c r="P40" s="36"/>
-      <c r="R40" s="75"/>
-      <c r="U40" s="75"/>
-      <c r="V40" s="76"/>
-    </row>
-    <row r="41" spans="1:22" ht="30.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="R40" s="73"/>
+      <c r="U40" s="73"/>
+      <c r="V40" s="74"/>
+    </row>
+    <row r="41" spans="1:22" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A41" s="1"/>
       <c r="B41" s="50">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>32</v>
       </c>
       <c r="C41" s="56" t="s">
@@ -3939,78 +3970,80 @@
         <v>1</v>
       </c>
       <c r="L41" s="38">
+        <f t="shared" si="2"/>
+        <v>10</v>
+      </c>
+      <c r="M41" s="38">
         <v>50</v>
       </c>
-      <c r="M41" s="62" t="s">
-        <v>341</v>
-      </c>
-      <c r="N41" s="63">
+      <c r="N41" s="61">
         <v>0.1096</v>
       </c>
-      <c r="O41" s="63">
-        <f t="shared" si="1"/>
+      <c r="O41" s="61">
+        <f t="shared" si="0"/>
         <v>5.48</v>
       </c>
       <c r="P41" s="38"/>
-      <c r="R41" s="75"/>
-      <c r="U41" s="75"/>
-      <c r="V41" s="76"/>
-    </row>
-    <row r="42" spans="1:22" ht="30.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="R41" s="73"/>
+      <c r="U41" s="73"/>
+      <c r="V41" s="74"/>
+    </row>
+    <row r="42" spans="1:22" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A42" s="1"/>
       <c r="B42" s="50">
         <f>ROW(B42) - ROW($B$9)</f>
         <v>33</v>
       </c>
-      <c r="C42" s="67" t="s">
+      <c r="C42" s="65" t="s">
         <v>312</v>
       </c>
-      <c r="D42" s="68" t="s">
+      <c r="D42" s="66" t="s">
         <v>39</v>
       </c>
-      <c r="E42" s="69" t="s">
+      <c r="E42" s="67" t="s">
         <v>107</v>
       </c>
-      <c r="F42" s="68" t="s">
+      <c r="F42" s="66" t="s">
         <v>304</v>
       </c>
-      <c r="G42" s="68" t="s">
+      <c r="G42" s="66" t="s">
         <v>161</v>
       </c>
-      <c r="H42" s="68" t="s">
+      <c r="H42" s="66" t="s">
         <v>243</v>
       </c>
-      <c r="I42" s="68" t="s">
-        <v>314</v>
-      </c>
-      <c r="J42" s="68" t="s">
-        <v>314</v>
-      </c>
-      <c r="K42" s="68">
+      <c r="I42" s="66" t="s">
+        <v>314</v>
+      </c>
+      <c r="J42" s="66" t="s">
+        <v>314</v>
+      </c>
+      <c r="K42" s="66">
         <v>4</v>
       </c>
-      <c r="L42" s="68">
+      <c r="L42" s="36">
+        <f t="shared" si="2"/>
+        <v>40</v>
+      </c>
+      <c r="M42" s="66">
         <v>80</v>
       </c>
-      <c r="M42" s="60" t="s">
-        <v>341</v>
-      </c>
-      <c r="N42" s="73">
+      <c r="N42" s="71">
         <v>3</v>
       </c>
-      <c r="O42" s="73">
-        <f t="shared" si="1"/>
+      <c r="O42" s="71">
+        <f t="shared" si="0"/>
         <v>240</v>
       </c>
       <c r="P42" s="36"/>
-      <c r="R42" s="75"/>
-      <c r="U42" s="75"/>
-      <c r="V42" s="76"/>
-    </row>
-    <row r="43" spans="1:22" ht="30.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="R42" s="73"/>
+      <c r="U42" s="73"/>
+      <c r="V42" s="74"/>
+    </row>
+    <row r="43" spans="1:22" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A43" s="1"/>
       <c r="B43" s="50">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>34</v>
       </c>
       <c r="C43" s="56" t="s">
@@ -4041,24 +4074,25 @@
         <v>4</v>
       </c>
       <c r="L43" s="38">
+        <f t="shared" si="2"/>
+        <v>40</v>
+      </c>
+      <c r="M43" s="38">
         <v>50</v>
       </c>
-      <c r="M43" s="62" t="s">
-        <v>341</v>
-      </c>
-      <c r="N43" s="63">
+      <c r="N43" s="61">
         <v>0.114</v>
       </c>
-      <c r="O43" s="63">
-        <f t="shared" si="1"/>
+      <c r="O43" s="61">
+        <f t="shared" si="0"/>
         <v>5.7</v>
       </c>
       <c r="P43" s="38"/>
-      <c r="R43" s="75"/>
-      <c r="U43" s="75"/>
-      <c r="V43" s="76"/>
-    </row>
-    <row r="44" spans="1:22" ht="30.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="R43" s="73"/>
+      <c r="U43" s="73"/>
+      <c r="V43" s="74"/>
+    </row>
+    <row r="44" spans="1:22" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A44" s="1"/>
       <c r="B44" s="50">
         <f>ROW(B44) - ROW($B$9)</f>
@@ -4092,27 +4126,28 @@
         <v>1</v>
       </c>
       <c r="L44" s="36">
+        <f t="shared" si="2"/>
+        <v>10</v>
+      </c>
+      <c r="M44" s="36">
         <v>20</v>
       </c>
-      <c r="M44" s="60" t="s">
-        <v>341</v>
-      </c>
-      <c r="N44" s="61">
+      <c r="N44" s="60">
         <v>0.13150000000000001</v>
       </c>
-      <c r="O44" s="61">
-        <f t="shared" si="1"/>
+      <c r="O44" s="60">
+        <f t="shared" si="0"/>
         <v>2.63</v>
       </c>
       <c r="P44" s="36"/>
-      <c r="R44" s="75"/>
-      <c r="U44" s="75"/>
-      <c r="V44" s="76"/>
+      <c r="R44" s="73"/>
+      <c r="U44" s="73"/>
+      <c r="V44" s="74"/>
     </row>
     <row r="45" spans="1:22" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A45" s="1"/>
       <c r="B45" s="50">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>36</v>
       </c>
       <c r="C45" s="56" t="s">
@@ -4142,24 +4177,25 @@
       <c r="K45" s="38">
         <v>5</v>
       </c>
-      <c r="L45" s="38" t="s">
-        <v>314</v>
-      </c>
-      <c r="M45" s="62" t="s">
-        <v>314</v>
-      </c>
-      <c r="N45" s="63">
+      <c r="L45" s="38">
+        <f t="shared" si="2"/>
+        <v>50</v>
+      </c>
+      <c r="M45" s="38" t="s">
+        <v>314</v>
+      </c>
+      <c r="N45" s="61">
         <v>0</v>
       </c>
-      <c r="O45" s="63" t="s">
+      <c r="O45" s="61" t="s">
         <v>314</v>
       </c>
       <c r="P45" s="38"/>
-      <c r="R45" s="75"/>
-      <c r="U45" s="75"/>
-      <c r="V45" s="76"/>
-    </row>
-    <row r="46" spans="1:22" ht="30.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="R45" s="73"/>
+      <c r="U45" s="73"/>
+      <c r="V45" s="74"/>
+    </row>
+    <row r="46" spans="1:22" ht="24.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A46" s="1"/>
       <c r="B46" s="50">
         <f>ROW(B46) - ROW($B$9)</f>
@@ -4193,27 +4229,28 @@
         <v>11</v>
       </c>
       <c r="L46" s="36">
+        <f t="shared" si="2"/>
+        <v>110</v>
+      </c>
+      <c r="M46" s="36">
         <v>200</v>
       </c>
-      <c r="M46" s="60" t="s">
-        <v>341</v>
-      </c>
-      <c r="N46" s="61">
+      <c r="N46" s="60">
         <v>0.1017</v>
       </c>
-      <c r="O46" s="61">
-        <f t="shared" si="1"/>
+      <c r="O46" s="60">
+        <f t="shared" ref="O46:O62" si="3">N46*M46</f>
         <v>20.34</v>
       </c>
       <c r="P46" s="36"/>
-      <c r="R46" s="75"/>
-      <c r="U46" s="75"/>
-      <c r="V46" s="76"/>
+      <c r="R46" s="73"/>
+      <c r="U46" s="73"/>
+      <c r="V46" s="74"/>
     </row>
     <row r="47" spans="1:22" ht="36.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A47" s="1"/>
       <c r="B47" s="50">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>38</v>
       </c>
       <c r="C47" s="56" t="s">
@@ -4244,24 +4281,25 @@
         <v>1</v>
       </c>
       <c r="L47" s="38">
+        <f t="shared" si="2"/>
+        <v>10</v>
+      </c>
+      <c r="M47" s="38">
         <v>50</v>
       </c>
-      <c r="M47" s="62" t="s">
-        <v>341</v>
-      </c>
-      <c r="N47" s="63">
+      <c r="N47" s="61">
         <v>0.10410000000000001</v>
       </c>
-      <c r="O47" s="63">
-        <f t="shared" si="1"/>
+      <c r="O47" s="61">
+        <f t="shared" si="3"/>
         <v>5.205000000000001</v>
       </c>
       <c r="P47" s="38"/>
-      <c r="R47" s="75"/>
-      <c r="U47" s="75"/>
-      <c r="V47" s="76"/>
-    </row>
-    <row r="48" spans="1:22" ht="30.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="R47" s="73"/>
+      <c r="U47" s="73"/>
+      <c r="V47" s="74"/>
+    </row>
+    <row r="48" spans="1:22" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A48" s="1"/>
       <c r="B48" s="50">
         <f>ROW(B48) - ROW($B$9)</f>
@@ -4295,27 +4333,28 @@
         <v>2</v>
       </c>
       <c r="L48" s="36">
+        <f t="shared" si="2"/>
+        <v>20</v>
+      </c>
+      <c r="M48" s="36">
         <v>100</v>
       </c>
-      <c r="M48" s="60" t="s">
-        <v>341</v>
-      </c>
-      <c r="N48" s="61">
+      <c r="N48" s="60">
         <v>0.1014</v>
       </c>
-      <c r="O48" s="61">
-        <f t="shared" si="1"/>
+      <c r="O48" s="60">
+        <f t="shared" si="3"/>
         <v>10.14</v>
       </c>
       <c r="P48" s="36"/>
-      <c r="R48" s="75"/>
-      <c r="U48" s="75"/>
-      <c r="V48" s="76"/>
-    </row>
-    <row r="49" spans="1:22" ht="30.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="R48" s="73"/>
+      <c r="U48" s="73"/>
+      <c r="V48" s="74"/>
+    </row>
+    <row r="49" spans="1:22" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A49" s="1"/>
       <c r="B49" s="50">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>40</v>
       </c>
       <c r="C49" s="56" t="s">
@@ -4346,22 +4385,23 @@
         <v>1</v>
       </c>
       <c r="L49" s="38">
+        <f t="shared" si="2"/>
+        <v>10</v>
+      </c>
+      <c r="M49" s="38">
         <v>100</v>
       </c>
-      <c r="M49" s="62" t="s">
-        <v>341</v>
-      </c>
-      <c r="N49" s="63">
+      <c r="N49" s="61">
         <v>0.1022</v>
       </c>
-      <c r="O49" s="63">
-        <f t="shared" si="1"/>
+      <c r="O49" s="61">
+        <f t="shared" si="3"/>
         <v>10.220000000000001</v>
       </c>
       <c r="P49" s="38"/>
-      <c r="R49" s="75"/>
-      <c r="U49" s="75"/>
-      <c r="V49" s="76"/>
+      <c r="R49" s="73"/>
+      <c r="U49" s="73"/>
+      <c r="V49" s="74"/>
     </row>
     <row r="50" spans="1:22" ht="36.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A50" s="1"/>
@@ -4397,27 +4437,28 @@
         <v>1</v>
       </c>
       <c r="L50" s="36">
+        <f t="shared" si="2"/>
+        <v>10</v>
+      </c>
+      <c r="M50" s="36">
         <v>20</v>
       </c>
-      <c r="M50" s="60" t="s">
-        <v>341</v>
-      </c>
-      <c r="N50" s="61">
+      <c r="N50" s="60">
         <v>0.1255</v>
       </c>
-      <c r="O50" s="61">
-        <f t="shared" si="1"/>
+      <c r="O50" s="60">
+        <f t="shared" si="3"/>
         <v>2.5099999999999998</v>
       </c>
       <c r="P50" s="36"/>
-      <c r="R50" s="75"/>
-      <c r="U50" s="75"/>
-      <c r="V50" s="76"/>
-    </row>
-    <row r="51" spans="1:22" ht="30.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="R50" s="73"/>
+      <c r="U50" s="73"/>
+      <c r="V50" s="74"/>
+    </row>
+    <row r="51" spans="1:22" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A51" s="1"/>
       <c r="B51" s="50">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>42</v>
       </c>
       <c r="C51" s="56" t="s">
@@ -4448,24 +4489,25 @@
         <v>1</v>
       </c>
       <c r="L51" s="38">
+        <f t="shared" si="2"/>
+        <v>10</v>
+      </c>
+      <c r="M51" s="38">
         <v>100</v>
       </c>
-      <c r="M51" s="62" t="s">
-        <v>341</v>
-      </c>
-      <c r="N51" s="63">
+      <c r="N51" s="61">
         <v>0.10150000000000001</v>
       </c>
-      <c r="O51" s="63">
-        <f t="shared" si="1"/>
+      <c r="O51" s="61">
+        <f t="shared" si="3"/>
         <v>10.15</v>
       </c>
       <c r="P51" s="38"/>
-      <c r="R51" s="75"/>
-      <c r="U51" s="75"/>
-      <c r="V51" s="76"/>
-    </row>
-    <row r="52" spans="1:22" ht="30.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="R51" s="73"/>
+      <c r="U51" s="73"/>
+      <c r="V51" s="74"/>
+    </row>
+    <row r="52" spans="1:22" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A52" s="1"/>
       <c r="B52" s="50">
         <f>ROW(B52) - ROW($B$9)</f>
@@ -4499,27 +4541,28 @@
         <v>1</v>
       </c>
       <c r="L52" s="36">
+        <f t="shared" si="2"/>
+        <v>10</v>
+      </c>
+      <c r="M52" s="36">
         <v>20</v>
       </c>
-      <c r="M52" s="60" t="s">
-        <v>341</v>
-      </c>
-      <c r="N52" s="61">
+      <c r="N52" s="60">
         <v>0.1376</v>
       </c>
-      <c r="O52" s="61">
-        <f t="shared" si="1"/>
+      <c r="O52" s="60">
+        <f t="shared" si="3"/>
         <v>2.7519999999999998</v>
       </c>
       <c r="P52" s="36"/>
-      <c r="R52" s="75"/>
-      <c r="U52" s="75"/>
-      <c r="V52" s="76"/>
-    </row>
-    <row r="53" spans="1:22" ht="30.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="R52" s="73"/>
+      <c r="U52" s="73"/>
+      <c r="V52" s="74"/>
+    </row>
+    <row r="53" spans="1:22" ht="24.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A53" s="1"/>
       <c r="B53" s="50">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>44</v>
       </c>
       <c r="C53" s="56" t="s">
@@ -4550,24 +4593,25 @@
         <v>1</v>
       </c>
       <c r="L53" s="38">
+        <f t="shared" si="2"/>
+        <v>10</v>
+      </c>
+      <c r="M53" s="38">
         <v>100</v>
       </c>
-      <c r="M53" s="62" t="s">
-        <v>341</v>
-      </c>
-      <c r="N53" s="63">
+      <c r="N53" s="61">
         <v>0.1018</v>
       </c>
-      <c r="O53" s="63">
-        <f t="shared" si="1"/>
+      <c r="O53" s="61">
+        <f t="shared" si="3"/>
         <v>10.18</v>
       </c>
       <c r="P53" s="38"/>
-      <c r="R53" s="75"/>
-      <c r="U53" s="75"/>
-      <c r="V53" s="76"/>
-    </row>
-    <row r="54" spans="1:22" ht="30.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="R53" s="73"/>
+      <c r="U53" s="73"/>
+      <c r="V53" s="74"/>
+    </row>
+    <row r="54" spans="1:22" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A54" s="1"/>
       <c r="B54" s="50">
         <f>ROW(B54) - ROW($B$9)</f>
@@ -4601,27 +4645,28 @@
         <v>2</v>
       </c>
       <c r="L54" s="36">
+        <f t="shared" si="2"/>
+        <v>20</v>
+      </c>
+      <c r="M54" s="36">
         <v>100</v>
       </c>
-      <c r="M54" s="60" t="s">
-        <v>341</v>
-      </c>
-      <c r="N54" s="61">
+      <c r="N54" s="60">
         <v>0.1013</v>
       </c>
-      <c r="O54" s="61">
-        <f t="shared" si="1"/>
+      <c r="O54" s="60">
+        <f t="shared" si="3"/>
         <v>10.130000000000001</v>
       </c>
       <c r="P54" s="36"/>
-      <c r="R54" s="75"/>
-      <c r="U54" s="75"/>
-      <c r="V54" s="76"/>
-    </row>
-    <row r="55" spans="1:22" ht="30.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="R54" s="73"/>
+      <c r="U54" s="73"/>
+      <c r="V54" s="74"/>
+    </row>
+    <row r="55" spans="1:22" ht="24.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A55" s="1"/>
       <c r="B55" s="50">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>46</v>
       </c>
       <c r="C55" s="56" t="s">
@@ -4652,24 +4697,25 @@
         <v>1</v>
       </c>
       <c r="L55" s="38">
+        <f t="shared" si="2"/>
+        <v>10</v>
+      </c>
+      <c r="M55" s="38">
         <v>100</v>
       </c>
-      <c r="M55" s="62" t="s">
-        <v>341</v>
-      </c>
-      <c r="N55" s="63">
+      <c r="N55" s="61">
         <v>0.1013</v>
       </c>
-      <c r="O55" s="63">
-        <f t="shared" si="1"/>
+      <c r="O55" s="61">
+        <f t="shared" si="3"/>
         <v>10.130000000000001</v>
       </c>
       <c r="P55" s="38"/>
-      <c r="R55" s="75"/>
-      <c r="U55" s="75"/>
-      <c r="V55" s="76"/>
-    </row>
-    <row r="56" spans="1:22" ht="30.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="R55" s="73"/>
+      <c r="U55" s="73"/>
+      <c r="V55" s="74"/>
+    </row>
+    <row r="56" spans="1:22" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A56" s="1"/>
       <c r="B56" s="50">
         <f>ROW(B56) - ROW($B$9)</f>
@@ -4703,34 +4749,35 @@
         <v>1</v>
       </c>
       <c r="L56" s="36">
+        <f t="shared" si="2"/>
+        <v>10</v>
+      </c>
+      <c r="M56" s="36">
         <v>100</v>
       </c>
-      <c r="M56" s="60" t="s">
-        <v>341</v>
-      </c>
-      <c r="N56" s="61">
+      <c r="N56" s="60">
         <v>0.1014</v>
       </c>
-      <c r="O56" s="61">
-        <f t="shared" si="1"/>
+      <c r="O56" s="60">
+        <f t="shared" si="3"/>
         <v>10.14</v>
       </c>
       <c r="P56" s="36"/>
-      <c r="R56" s="75"/>
-      <c r="U56" s="75"/>
-      <c r="V56" s="76"/>
-    </row>
-    <row r="57" spans="1:22" ht="30.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="R56" s="73"/>
+      <c r="U56" s="73"/>
+      <c r="V56" s="74"/>
+    </row>
+    <row r="57" spans="1:22" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A57" s="1"/>
       <c r="B57" s="50">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>48</v>
       </c>
       <c r="C57" s="56" t="s">
         <v>315</v>
       </c>
       <c r="D57" s="38" t="s">
-        <v>345</v>
+        <v>343</v>
       </c>
       <c r="E57" s="39" t="s">
         <v>122</v>
@@ -4754,24 +4801,25 @@
         <v>2</v>
       </c>
       <c r="L57" s="38">
+        <f t="shared" si="2"/>
+        <v>20</v>
+      </c>
+      <c r="M57" s="38">
         <v>40</v>
       </c>
-      <c r="M57" s="62" t="s">
-        <v>341</v>
-      </c>
-      <c r="N57" s="63">
+      <c r="N57" s="61">
         <v>0.13290000000000002</v>
       </c>
-      <c r="O57" s="63">
-        <f t="shared" si="1"/>
+      <c r="O57" s="61">
+        <f t="shared" si="3"/>
         <v>5.3160000000000007</v>
       </c>
       <c r="P57" s="38"/>
-      <c r="R57" s="75"/>
-      <c r="U57" s="75"/>
-      <c r="V57" s="76"/>
-    </row>
-    <row r="58" spans="1:22" ht="30.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="R57" s="73"/>
+      <c r="U57" s="73"/>
+      <c r="V57" s="74"/>
+    </row>
+    <row r="58" spans="1:22" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A58" s="1"/>
       <c r="B58" s="50">
         <f>ROW(B58) - ROW($B$9)</f>
@@ -4805,27 +4853,28 @@
         <v>4</v>
       </c>
       <c r="L58" s="36">
+        <f t="shared" si="2"/>
+        <v>40</v>
+      </c>
+      <c r="M58" s="36">
         <v>50</v>
       </c>
-      <c r="M58" s="60" t="s">
-        <v>341</v>
-      </c>
-      <c r="N58" s="61">
+      <c r="N58" s="60">
         <v>0.1072</v>
       </c>
-      <c r="O58" s="61">
-        <f t="shared" si="1"/>
+      <c r="O58" s="60">
+        <f t="shared" si="3"/>
         <v>5.36</v>
       </c>
       <c r="P58" s="36"/>
-      <c r="R58" s="75"/>
-      <c r="U58" s="75"/>
-      <c r="V58" s="76"/>
-    </row>
-    <row r="59" spans="1:22" ht="30.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="R58" s="73"/>
+      <c r="U58" s="73"/>
+      <c r="V58" s="74"/>
+    </row>
+    <row r="59" spans="1:22" ht="24.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A59" s="1"/>
       <c r="B59" s="50">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>50</v>
       </c>
       <c r="C59" s="56" t="s">
@@ -4854,24 +4903,25 @@
         <v>2</v>
       </c>
       <c r="L59" s="38">
+        <f t="shared" si="2"/>
+        <v>20</v>
+      </c>
+      <c r="M59" s="38">
         <v>40</v>
       </c>
-      <c r="M59" s="62" t="s">
-        <v>341</v>
-      </c>
-      <c r="N59" s="63">
+      <c r="N59" s="61">
         <v>0.13550000000000001</v>
       </c>
-      <c r="O59" s="63">
-        <f t="shared" si="1"/>
+      <c r="O59" s="61">
+        <f t="shared" si="3"/>
         <v>5.42</v>
       </c>
       <c r="P59" s="38"/>
-      <c r="R59" s="75"/>
-      <c r="U59" s="75"/>
-      <c r="V59" s="76"/>
-    </row>
-    <row r="60" spans="1:22" ht="30.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="R59" s="73"/>
+      <c r="U59" s="73"/>
+      <c r="V59" s="74"/>
+    </row>
+    <row r="60" spans="1:22" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A60" s="1"/>
       <c r="B60" s="50">
         <f>ROW(B60) - ROW($B$9)</f>
@@ -4905,27 +4955,28 @@
         <v>1</v>
       </c>
       <c r="L60" s="36">
+        <f t="shared" si="2"/>
+        <v>10</v>
+      </c>
+      <c r="M60" s="36">
         <v>20</v>
       </c>
-      <c r="M60" s="60" t="s">
-        <v>341</v>
-      </c>
-      <c r="N60" s="61">
+      <c r="N60" s="60">
         <v>0.1391</v>
       </c>
-      <c r="O60" s="61">
-        <f t="shared" si="1"/>
+      <c r="O60" s="60">
+        <f t="shared" si="3"/>
         <v>2.782</v>
       </c>
       <c r="P60" s="36"/>
-      <c r="R60" s="75"/>
-      <c r="U60" s="75"/>
-      <c r="V60" s="76"/>
-    </row>
-    <row r="61" spans="1:22" ht="30.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="R60" s="73"/>
+      <c r="U60" s="73"/>
+      <c r="V60" s="74"/>
+    </row>
+    <row r="61" spans="1:22" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A61" s="1"/>
       <c r="B61" s="50">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>52</v>
       </c>
       <c r="C61" s="56" t="s">
@@ -4954,24 +5005,25 @@
         <v>1</v>
       </c>
       <c r="L61" s="38">
+        <f t="shared" si="2"/>
+        <v>10</v>
+      </c>
+      <c r="M61" s="38">
         <v>50</v>
       </c>
-      <c r="M61" s="62" t="s">
-        <v>341</v>
-      </c>
-      <c r="N61" s="63">
+      <c r="N61" s="61">
         <v>0.11430000000000001</v>
       </c>
-      <c r="O61" s="63">
-        <f t="shared" si="1"/>
+      <c r="O61" s="61">
+        <f t="shared" si="3"/>
         <v>5.7150000000000007</v>
       </c>
       <c r="P61" s="38"/>
-      <c r="R61" s="75"/>
-      <c r="U61" s="75"/>
-      <c r="V61" s="76"/>
-    </row>
-    <row r="62" spans="1:22" ht="30.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="R61" s="73"/>
+      <c r="U61" s="73"/>
+      <c r="V61" s="74"/>
+    </row>
+    <row r="62" spans="1:22" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A62" s="1"/>
       <c r="B62" s="50">
         <f>ROW(B62) - ROW($B$9)</f>
@@ -5003,27 +5055,28 @@
         <v>2</v>
       </c>
       <c r="L62" s="36">
+        <f t="shared" si="2"/>
+        <v>20</v>
+      </c>
+      <c r="M62" s="36">
         <v>100</v>
       </c>
-      <c r="M62" s="60" t="s">
-        <v>341</v>
-      </c>
-      <c r="N62" s="61">
+      <c r="N62" s="60">
         <v>0.10100000000000001</v>
       </c>
-      <c r="O62" s="61">
-        <f t="shared" si="1"/>
+      <c r="O62" s="60">
+        <f t="shared" si="3"/>
         <v>10.100000000000001</v>
       </c>
       <c r="P62" s="36"/>
-      <c r="R62" s="75"/>
-      <c r="U62" s="75"/>
-      <c r="V62" s="76"/>
+      <c r="R62" s="73"/>
+      <c r="U62" s="73"/>
+      <c r="V62" s="74"/>
     </row>
     <row r="63" spans="1:22" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A63" s="1"/>
       <c r="B63" s="50">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>54</v>
       </c>
       <c r="C63" s="56" t="s">
@@ -5053,22 +5106,23 @@
       <c r="K63" s="38">
         <v>9</v>
       </c>
-      <c r="L63" s="38" t="s">
-        <v>314</v>
-      </c>
-      <c r="M63" s="62" t="s">
-        <v>314</v>
-      </c>
-      <c r="N63" s="63">
+      <c r="L63" s="38">
+        <f t="shared" si="2"/>
+        <v>90</v>
+      </c>
+      <c r="M63" s="38" t="s">
+        <v>314</v>
+      </c>
+      <c r="N63" s="61">
         <v>0</v>
       </c>
-      <c r="O63" s="63" t="s">
+      <c r="O63" s="61" t="s">
         <v>314</v>
       </c>
       <c r="P63" s="38"/>
-      <c r="R63" s="75"/>
-      <c r="U63" s="75"/>
-      <c r="V63" s="76"/>
+      <c r="R63" s="73"/>
+      <c r="U63" s="73"/>
+      <c r="V63" s="74"/>
     </row>
     <row r="64" spans="1:22" ht="36.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A64" s="1"/>
@@ -5104,27 +5158,28 @@
         <v>1</v>
       </c>
       <c r="L64" s="36">
+        <f t="shared" si="2"/>
+        <v>10</v>
+      </c>
+      <c r="M64" s="36">
         <v>20</v>
       </c>
-      <c r="M64" s="60" t="s">
-        <v>341</v>
-      </c>
-      <c r="N64" s="61">
+      <c r="N64" s="60">
         <v>0.16189999999999999</v>
       </c>
-      <c r="O64" s="61">
-        <f t="shared" si="1"/>
+      <c r="O64" s="60">
+        <f t="shared" ref="O64:O77" si="4">N64*M64</f>
         <v>3.2379999999999995</v>
       </c>
       <c r="P64" s="36"/>
-      <c r="R64" s="75"/>
-      <c r="U64" s="75"/>
-      <c r="V64" s="76"/>
-    </row>
-    <row r="65" spans="1:22" ht="30.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="R64" s="73"/>
+      <c r="U64" s="73"/>
+      <c r="V64" s="74"/>
+    </row>
+    <row r="65" spans="1:22" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A65" s="1"/>
       <c r="B65" s="50">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>56</v>
       </c>
       <c r="C65" s="56" t="s">
@@ -5155,24 +5210,25 @@
         <v>1</v>
       </c>
       <c r="L65" s="38">
+        <f t="shared" si="2"/>
+        <v>10</v>
+      </c>
+      <c r="M65" s="38">
         <v>11</v>
       </c>
-      <c r="M65" s="62" t="s">
-        <v>341</v>
-      </c>
-      <c r="N65" s="63">
+      <c r="N65" s="61">
         <v>2.0760999999999998</v>
       </c>
-      <c r="O65" s="63">
-        <f t="shared" si="1"/>
+      <c r="O65" s="61">
+        <f t="shared" si="4"/>
         <v>22.8371</v>
       </c>
       <c r="P65" s="38"/>
-      <c r="R65" s="75"/>
-      <c r="U65" s="75"/>
-      <c r="V65" s="76"/>
-    </row>
-    <row r="66" spans="1:22" ht="30.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="R65" s="73"/>
+      <c r="U65" s="73"/>
+      <c r="V65" s="74"/>
+    </row>
+    <row r="66" spans="1:22" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A66" s="1"/>
       <c r="B66" s="50">
         <f>ROW(B66) - ROW($B$9)</f>
@@ -5206,27 +5262,28 @@
         <v>1</v>
       </c>
       <c r="L66" s="36">
+        <f t="shared" si="2"/>
+        <v>10</v>
+      </c>
+      <c r="M66" s="36">
         <v>11</v>
       </c>
-      <c r="M66" s="60" t="s">
-        <v>341</v>
-      </c>
-      <c r="N66" s="61">
+      <c r="N66" s="60">
         <v>0.52690000000000003</v>
       </c>
-      <c r="O66" s="61">
-        <f t="shared" si="1"/>
+      <c r="O66" s="60">
+        <f t="shared" si="4"/>
         <v>5.7959000000000005</v>
       </c>
       <c r="P66" s="36"/>
-      <c r="R66" s="75"/>
-      <c r="U66" s="75"/>
-      <c r="V66" s="76"/>
-    </row>
-    <row r="67" spans="1:22" ht="30.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="R66" s="73"/>
+      <c r="U66" s="73"/>
+      <c r="V66" s="74"/>
+    </row>
+    <row r="67" spans="1:22" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A67" s="1"/>
       <c r="B67" s="50">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>58</v>
       </c>
       <c r="C67" s="56" t="s">
@@ -5257,24 +5314,25 @@
         <v>1</v>
       </c>
       <c r="L67" s="38">
+        <f t="shared" si="2"/>
+        <v>10</v>
+      </c>
+      <c r="M67" s="38">
         <v>11</v>
       </c>
-      <c r="M67" s="62" t="s">
-        <v>341</v>
-      </c>
-      <c r="N67" s="63">
+      <c r="N67" s="61">
         <v>0.54239999999999999</v>
       </c>
-      <c r="O67" s="63">
-        <f t="shared" si="1"/>
+      <c r="O67" s="61">
+        <f t="shared" si="4"/>
         <v>5.9664000000000001</v>
       </c>
       <c r="P67" s="38"/>
-      <c r="R67" s="75"/>
-      <c r="U67" s="75"/>
-      <c r="V67" s="76"/>
-    </row>
-    <row r="68" spans="1:22" ht="30.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="R67" s="73"/>
+      <c r="U67" s="73"/>
+      <c r="V67" s="74"/>
+    </row>
+    <row r="68" spans="1:22" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A68" s="1"/>
       <c r="B68" s="50">
         <f>ROW(B68) - ROW($B$9)</f>
@@ -5308,27 +5366,28 @@
         <v>1</v>
       </c>
       <c r="L68" s="36">
+        <f t="shared" si="2"/>
+        <v>10</v>
+      </c>
+      <c r="M68" s="36">
         <v>11</v>
       </c>
-      <c r="M68" s="60" t="s">
-        <v>341</v>
-      </c>
-      <c r="N68" s="61">
+      <c r="N68" s="60">
         <v>1.7232000000000001</v>
       </c>
-      <c r="O68" s="61">
-        <f t="shared" si="1"/>
+      <c r="O68" s="60">
+        <f t="shared" si="4"/>
         <v>18.955200000000001</v>
       </c>
       <c r="P68" s="36"/>
-      <c r="R68" s="75"/>
-      <c r="U68" s="75"/>
-      <c r="V68" s="76"/>
+      <c r="R68" s="73"/>
+      <c r="U68" s="73"/>
+      <c r="V68" s="74"/>
     </row>
     <row r="69" spans="1:22" ht="36.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A69" s="1"/>
       <c r="B69" s="50">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>60</v>
       </c>
       <c r="C69" s="56" t="s">
@@ -5359,24 +5418,25 @@
         <v>1</v>
       </c>
       <c r="L69" s="38">
+        <f t="shared" si="2"/>
+        <v>10</v>
+      </c>
+      <c r="M69" s="38">
         <v>20</v>
       </c>
-      <c r="M69" s="62" t="s">
-        <v>341</v>
-      </c>
-      <c r="N69" s="63">
+      <c r="N69" s="61">
         <v>0.15640000000000001</v>
       </c>
-      <c r="O69" s="63">
-        <f t="shared" si="1"/>
+      <c r="O69" s="61">
+        <f t="shared" si="4"/>
         <v>3.1280000000000001</v>
       </c>
       <c r="P69" s="38"/>
-      <c r="R69" s="75"/>
-      <c r="U69" s="75"/>
-      <c r="V69" s="76"/>
-    </row>
-    <row r="70" spans="1:22" ht="30.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="R69" s="73"/>
+      <c r="U69" s="73"/>
+      <c r="V69" s="74"/>
+    </row>
+    <row r="70" spans="1:22" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A70" s="1"/>
       <c r="B70" s="50">
         <f>ROW(B70) - ROW($B$9)</f>
@@ -5410,27 +5470,28 @@
         <v>1</v>
       </c>
       <c r="L70" s="36">
+        <f t="shared" si="2"/>
+        <v>10</v>
+      </c>
+      <c r="M70" s="36">
         <v>11</v>
       </c>
-      <c r="M70" s="60" t="s">
-        <v>341</v>
-      </c>
-      <c r="N70" s="61">
+      <c r="N70" s="60">
         <v>4.0366999999999997</v>
       </c>
-      <c r="O70" s="61">
-        <f t="shared" si="1"/>
+      <c r="O70" s="60">
+        <f t="shared" si="4"/>
         <v>44.403700000000001</v>
       </c>
       <c r="P70" s="36"/>
-      <c r="R70" s="75"/>
-      <c r="U70" s="75"/>
-      <c r="V70" s="76"/>
-    </row>
-    <row r="71" spans="1:22" ht="30.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="R70" s="73"/>
+      <c r="U70" s="73"/>
+      <c r="V70" s="74"/>
+    </row>
+    <row r="71" spans="1:22" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A71" s="1"/>
       <c r="B71" s="50">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>62</v>
       </c>
       <c r="C71" s="56" t="s">
@@ -5461,24 +5522,25 @@
         <v>1</v>
       </c>
       <c r="L71" s="38">
+        <f t="shared" si="2"/>
+        <v>10</v>
+      </c>
+      <c r="M71" s="38">
         <v>11</v>
       </c>
-      <c r="M71" s="62" t="s">
-        <v>341</v>
-      </c>
-      <c r="N71" s="63">
+      <c r="N71" s="61">
         <v>1.0433000000000001</v>
       </c>
-      <c r="O71" s="63">
-        <f t="shared" si="1"/>
+      <c r="O71" s="61">
+        <f t="shared" si="4"/>
         <v>11.476300000000002</v>
       </c>
       <c r="P71" s="38"/>
-      <c r="R71" s="75"/>
-      <c r="U71" s="75"/>
-      <c r="V71" s="76"/>
-    </row>
-    <row r="72" spans="1:22" ht="30.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="R71" s="73"/>
+      <c r="U71" s="73"/>
+      <c r="V71" s="74"/>
+    </row>
+    <row r="72" spans="1:22" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A72" s="1"/>
       <c r="B72" s="50">
         <f>ROW(B72) - ROW($B$9)</f>
@@ -5512,27 +5574,28 @@
         <v>1</v>
       </c>
       <c r="L72" s="36">
+        <f t="shared" si="2"/>
+        <v>10</v>
+      </c>
+      <c r="M72" s="36">
         <v>11</v>
       </c>
-      <c r="M72" s="60" t="s">
-        <v>341</v>
-      </c>
-      <c r="N72" s="61">
+      <c r="N72" s="60">
         <v>0.82819999999999994</v>
       </c>
-      <c r="O72" s="61">
-        <f t="shared" si="1"/>
+      <c r="O72" s="60">
+        <f t="shared" si="4"/>
         <v>9.110199999999999</v>
       </c>
       <c r="P72" s="36"/>
-      <c r="R72" s="75"/>
-      <c r="U72" s="75"/>
-      <c r="V72" s="76"/>
-    </row>
-    <row r="73" spans="1:22" ht="30.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="R72" s="73"/>
+      <c r="U72" s="73"/>
+      <c r="V72" s="74"/>
+    </row>
+    <row r="73" spans="1:22" ht="24.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A73" s="1"/>
       <c r="B73" s="50">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>64</v>
       </c>
       <c r="C73" s="56" t="s">
@@ -5563,122 +5626,125 @@
         <v>1</v>
       </c>
       <c r="L73" s="38">
+        <f t="shared" si="2"/>
+        <v>10</v>
+      </c>
+      <c r="M73" s="38">
         <v>11</v>
       </c>
-      <c r="M73" s="62" t="s">
-        <v>341</v>
-      </c>
-      <c r="N73" s="63">
+      <c r="N73" s="61">
         <v>1.4220000000000002</v>
       </c>
-      <c r="O73" s="63">
-        <f t="shared" si="1"/>
+      <c r="O73" s="61">
+        <f t="shared" si="4"/>
         <v>15.642000000000001</v>
       </c>
       <c r="P73" s="38"/>
-      <c r="R73" s="75"/>
-      <c r="U73" s="75"/>
-      <c r="V73" s="76"/>
-    </row>
-    <row r="74" spans="1:22" ht="30.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="R73" s="73"/>
+      <c r="U73" s="73"/>
+      <c r="V73" s="74"/>
+    </row>
+    <row r="74" spans="1:22" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A74" s="1"/>
       <c r="B74" s="50">
         <f>ROW(B74) - ROW($B$9)</f>
         <v>65</v>
       </c>
-      <c r="C74" s="67" t="s">
+      <c r="C74" s="65" t="s">
         <v>320</v>
       </c>
-      <c r="D74" s="68" t="s">
+      <c r="D74" s="66" t="s">
         <v>70</v>
       </c>
-      <c r="E74" s="69" t="s">
+      <c r="E74" s="67" t="s">
         <v>139</v>
       </c>
-      <c r="F74" s="68" t="s">
+      <c r="F74" s="66" t="s">
         <v>304</v>
       </c>
-      <c r="G74" s="68" t="s">
+      <c r="G74" s="66" t="s">
         <v>179</v>
       </c>
-      <c r="H74" s="68" t="s">
+      <c r="H74" s="66" t="s">
         <v>254</v>
       </c>
       <c r="I74" s="59"/>
-      <c r="J74" s="68" t="s">
-        <v>314</v>
-      </c>
-      <c r="K74" s="68">
+      <c r="J74" s="66" t="s">
+        <v>314</v>
+      </c>
+      <c r="K74" s="66">
         <v>1</v>
       </c>
-      <c r="L74" s="68">
+      <c r="L74" s="36">
+        <f t="shared" si="2"/>
+        <v>10</v>
+      </c>
+      <c r="M74" s="66">
         <v>11</v>
       </c>
-      <c r="M74" s="60" t="s">
-        <v>341</v>
-      </c>
-      <c r="N74" s="73">
+      <c r="N74" s="71">
         <v>1.26</v>
       </c>
-      <c r="O74" s="73">
-        <f t="shared" si="1"/>
+      <c r="O74" s="71">
+        <f t="shared" si="4"/>
         <v>13.86</v>
       </c>
       <c r="P74" s="36"/>
-      <c r="R74" s="75"/>
-      <c r="U74" s="75"/>
-      <c r="V74" s="76"/>
-    </row>
-    <row r="75" spans="1:22" ht="30.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="R74" s="73"/>
+      <c r="U74" s="73"/>
+      <c r="V74" s="74"/>
+    </row>
+    <row r="75" spans="1:22" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A75" s="1"/>
       <c r="B75" s="50">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>66</v>
       </c>
-      <c r="C75" s="70" t="s">
+      <c r="C75" s="68" t="s">
         <v>320</v>
       </c>
-      <c r="D75" s="71" t="s">
+      <c r="D75" s="69" t="s">
         <v>71</v>
       </c>
-      <c r="E75" s="72" t="s">
+      <c r="E75" s="70" t="s">
         <v>140</v>
       </c>
-      <c r="F75" s="71" t="s">
+      <c r="F75" s="69" t="s">
         <v>171</v>
       </c>
       <c r="G75" s="57">
         <v>4677</v>
       </c>
-      <c r="H75" s="71" t="s">
+      <c r="H75" s="69" t="s">
         <v>255</v>
       </c>
       <c r="I75" s="38" t="s">
-        <v>340</v>
-      </c>
-      <c r="J75" s="71" t="s">
-        <v>314</v>
-      </c>
-      <c r="K75" s="71">
+        <v>339</v>
+      </c>
+      <c r="J75" s="69" t="s">
+        <v>314</v>
+      </c>
+      <c r="K75" s="69">
         <v>1</v>
       </c>
-      <c r="L75" s="71">
+      <c r="L75" s="38">
+        <f t="shared" ref="L75:L77" si="5">K75*10</f>
+        <v>10</v>
+      </c>
+      <c r="M75" s="69">
         <v>11</v>
       </c>
-      <c r="M75" s="62" t="s">
-        <v>341</v>
-      </c>
-      <c r="N75" s="74">
+      <c r="N75" s="72">
         <v>2.8662000000000001</v>
       </c>
-      <c r="O75" s="74">
-        <f t="shared" ref="O75:O77" si="2">N75*L75</f>
+      <c r="O75" s="72">
+        <f t="shared" si="4"/>
         <v>31.528200000000002</v>
       </c>
       <c r="P75" s="38"/>
-      <c r="R75" s="75"/>
-      <c r="U75" s="75"/>
-      <c r="V75" s="76"/>
+      <c r="R75" s="73"/>
+      <c r="U75" s="73"/>
+      <c r="V75" s="74"/>
     </row>
     <row r="76" spans="1:22" ht="36.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A76" s="1"/>
@@ -5714,27 +5780,28 @@
         <v>1</v>
       </c>
       <c r="L76" s="36">
+        <f t="shared" si="5"/>
+        <v>10</v>
+      </c>
+      <c r="M76" s="36">
         <v>15</v>
       </c>
-      <c r="M76" s="60" t="s">
-        <v>341</v>
-      </c>
-      <c r="N76" s="61">
+      <c r="N76" s="60">
         <v>0.19</v>
       </c>
-      <c r="O76" s="61">
-        <f t="shared" si="2"/>
+      <c r="O76" s="60">
+        <f t="shared" si="4"/>
         <v>2.85</v>
       </c>
       <c r="P76" s="36"/>
-      <c r="R76" s="75"/>
-      <c r="U76" s="75"/>
-      <c r="V76" s="76"/>
+      <c r="R76" s="73"/>
+      <c r="U76" s="73"/>
+      <c r="V76" s="74"/>
     </row>
     <row r="77" spans="1:22" ht="36.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A77" s="1"/>
       <c r="B77" s="50">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>68</v>
       </c>
       <c r="C77" s="56" t="s">
@@ -5761,26 +5828,27 @@
       <c r="J77" s="38" t="s">
         <v>300</v>
       </c>
-      <c r="K77" s="66">
+      <c r="K77" s="64">
         <v>1</v>
       </c>
       <c r="L77" s="38">
+        <f t="shared" si="5"/>
+        <v>10</v>
+      </c>
+      <c r="M77" s="38">
         <v>15</v>
       </c>
-      <c r="M77" s="62" t="s">
-        <v>341</v>
-      </c>
-      <c r="N77" s="63">
+      <c r="N77" s="61">
         <v>0.16510000000000002</v>
       </c>
-      <c r="O77" s="63">
-        <f t="shared" si="2"/>
+      <c r="O77" s="61">
+        <f t="shared" si="4"/>
         <v>2.4765000000000006</v>
       </c>
       <c r="P77" s="38"/>
-      <c r="R77" s="75"/>
-      <c r="U77" s="75"/>
-      <c r="V77" s="76"/>
+      <c r="R77" s="73"/>
+      <c r="U77" s="73"/>
+      <c r="V77" s="74"/>
     </row>
     <row r="78" spans="1:22" ht="19.5" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A78" s="1"/>
@@ -5794,18 +5862,18 @@
       <c r="I78" s="34"/>
       <c r="J78" s="35"/>
       <c r="K78" s="35"/>
-      <c r="L78" s="80" t="s">
-        <v>338</v>
-      </c>
-      <c r="M78" s="81"/>
-      <c r="N78" s="81"/>
-      <c r="O78" s="64">
+      <c r="L78" s="35"/>
+      <c r="M78" s="79" t="s">
+        <v>337</v>
+      </c>
+      <c r="N78" s="80"/>
+      <c r="O78" s="62">
         <f>SUM(O10:O77)</f>
         <v>839.02409999999998</v>
       </c>
       <c r="P78" s="41"/>
-      <c r="U78" s="75"/>
-      <c r="V78" s="75"/>
+      <c r="U78" s="73"/>
+      <c r="V78" s="73"/>
     </row>
     <row r="79" spans="1:22" ht="19.5" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A79" s="1"/>
@@ -5819,26 +5887,26 @@
       <c r="I79" s="9"/>
       <c r="J79" s="9"/>
       <c r="K79" s="9"/>
-      <c r="L79" s="80" t="s">
-        <v>339</v>
-      </c>
-      <c r="M79" s="81"/>
-      <c r="N79" s="81"/>
-      <c r="O79" s="65">
+      <c r="L79" s="9"/>
+      <c r="M79" s="79" t="s">
+        <v>338</v>
+      </c>
+      <c r="N79" s="80"/>
+      <c r="O79" s="63">
         <f>O78/10</f>
         <v>83.902410000000003</v>
       </c>
       <c r="P79" s="42"/>
     </row>
     <row r="84" spans="14:14" x14ac:dyDescent="0.25">
-      <c r="N84" s="75"/>
+      <c r="N84" s="73"/>
     </row>
   </sheetData>
   <mergeCells count="4">
     <mergeCell ref="J1:P1"/>
     <mergeCell ref="P3:P8"/>
-    <mergeCell ref="L78:N78"/>
-    <mergeCell ref="L79:N79"/>
+    <mergeCell ref="M78:N78"/>
+    <mergeCell ref="M79:N79"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>

</xml_diff>